<commit_message>
added supplies for burning
</commit_message>
<xml_diff>
--- a/DFT_6311_Result.xlsx
+++ b/DFT_6311_Result.xlsx
@@ -457,7 +457,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>1.7984004575</v>
+        <v>1.7984258975</v>
       </c>
     </row>
     <row r="3">
@@ -472,7 +472,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0.541737476</v>
+        <v>0.5413890625</v>
       </c>
     </row>
     <row r="4">
@@ -487,7 +487,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>811247.5399999999</v>
+        <v>811252.135</v>
       </c>
     </row>
     <row r="5">
@@ -502,7 +502,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0.70363960275</v>
+        <v>0.70521880475</v>
       </c>
     </row>
     <row r="6">

</xml_diff>

<commit_message>
working on the boost
</commit_message>
<xml_diff>
--- a/DFT_6311_Result.xlsx
+++ b/DFT_6311_Result.xlsx
@@ -8,7 +8,6 @@
   </bookViews>
   <sheets>
     <sheet name="Trimming" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="AZ_comp" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -454,11 +453,11 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>AE</t>
+          <t>3E</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>1.80081047</v>
+        <v>1.796360665</v>
       </c>
     </row>
     <row r="3">
@@ -469,11 +468,11 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>DF</t>
+          <t>9F</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0.540902031</v>
+        <v>0.5395462332500001</v>
       </c>
     </row>
     <row r="4">
@@ -484,11 +483,11 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>E6</t>
+          <t>E5</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>810821.9599999997</v>
+        <v>812031.0349999997</v>
       </c>
     </row>
     <row r="5">
@@ -499,11 +498,11 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>7F</t>
+          <t>71</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0.7120892114999999</v>
+        <v>0.80392019</v>
       </c>
     </row>
     <row r="6">
@@ -514,105 +513,10 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>F0</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B8"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Row Name</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Measure Values</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>3rd_STG_Current</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>9.842110652499999e-07</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>2nd_STG_Current</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>1.4480021675e-06</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>1st_STG_Current</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>8.1009359825e-07</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Ground_AZCOMP</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>1.1971836e-05</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>OUTN_EXT_PRT</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>2.0038760375</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>OUTP_EXT_PRT</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>2.00630406</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>VCM_AVDD</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>1.80360095</v>
-      </c>
+          <t>D0</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
working on ocp trim, doesnt work well, 0x7f is not 0x7f but 0x70
</commit_message>
<xml_diff>
--- a/DFT_6311_Result.xlsx
+++ b/DFT_6311_Result.xlsx
@@ -453,11 +453,11 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>9E</t>
+          <t>8E</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>1.80113295</v>
+        <v>1.792773715</v>
       </c>
     </row>
     <row r="3">
@@ -468,11 +468,11 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>9F</t>
+          <t>7F</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0.5407040400000001</v>
+        <v>0.5447496152500001</v>
       </c>
     </row>
     <row r="4">
@@ -483,11 +483,11 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>F1</t>
+          <t>F3</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>806553.845</v>
+        <v>811697.5550000004</v>
       </c>
     </row>
     <row r="5">
@@ -498,11 +498,11 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>72</t>
+          <t>7F</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0.7674725210000001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">

</xml_diff>

<commit_message>
solve problem vbso must be 5V before was 3.6V, the chip didn't able to close the high side.Change, also, the DFT of 6311, set vbso to 5V
</commit_message>
<xml_diff>
--- a/DFT_6311_Result.xlsx
+++ b/DFT_6311_Result.xlsx
@@ -453,11 +453,11 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>8E</t>
+          <t>70</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>1.792773715</v>
+        <v>1.795640945</v>
       </c>
     </row>
     <row r="3">
@@ -468,12 +468,10 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>7F</t>
-        </is>
-      </c>
-      <c r="C3" t="n">
-        <v>0.5447496152500001</v>
-      </c>
+          <t>F0</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -481,14 +479,8 @@
           <t>FRO_CLOCK</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>F3</t>
-        </is>
-      </c>
-      <c r="C4" t="n">
-        <v>811697.5550000004</v>
-      </c>
+      <c r="B4" t="inlineStr"/>
+      <c r="C4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -496,14 +488,8 @@
           <t>BST_OCP_TRIM_reg1</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>7F</t>
-        </is>
-      </c>
-      <c r="C5" t="n">
-        <v>0</v>
-      </c>
+      <c r="B5" t="inlineStr"/>
+      <c r="C5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -511,11 +497,7 @@
           <t>BST_OCP_TRIM_reg2</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>D0</t>
-        </is>
-      </c>
+      <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
stable conditions. everythings is working, i will add zc_trim in the reference and some other tests and modify in boost, AZ_com is ok
</commit_message>
<xml_diff>
--- a/DFT_6311_Result.xlsx
+++ b/DFT_6311_Result.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="Trimming" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="AZ_comp" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -453,11 +454,11 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>70</t>
+          <t>8E</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>1.795640945</v>
+        <v>1.792584265</v>
       </c>
     </row>
     <row r="3">
@@ -468,10 +469,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>F0</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr"/>
+          <t>7F</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>0.5414111315</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -479,8 +482,14 @@
           <t>FRO_CLOCK</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr"/>
-      <c r="C4" t="inlineStr"/>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>E7</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>812153.6900000001</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -488,8 +497,14 @@
           <t>BST_OCP_TRIM_reg1</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr"/>
-      <c r="C5" t="inlineStr"/>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>1.7959239975</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -497,8 +512,107 @@
           <t>BST_OCP_TRIM_reg2</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr"/>
-      <c r="C6" t="inlineStr"/>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>F0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Row Name</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Measure Values</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>3rd_STG_Current</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>9.564949367500002e-07</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2nd_STG_Current</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>1.428297495e-06</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>1st_STG_Current</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>7.80791412e-07</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Ground_AZCOMP</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>1.08070087e-05</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>OUTN_EXT_PRT</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>2.0037971025</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>OUTP_EXT_PRT</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>2.0067665425</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>VCM_AVDD</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>1.80382072</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
modified reference script, after eaxh tests i write the trimming inside the right register
</commit_message>
<xml_diff>
--- a/DFT_6311_Result.xlsx
+++ b/DFT_6311_Result.xlsx
@@ -8,7 +8,6 @@
   </bookViews>
   <sheets>
     <sheet name="Trimming" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="AZ_comp" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -458,7 +457,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>1.792584265</v>
+        <v>1.80022254</v>
       </c>
     </row>
     <row r="3">
@@ -469,11 +468,11 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>7F</t>
+          <t>9F</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0.5414111315</v>
+        <v>0.5422006655</v>
       </c>
     </row>
     <row r="4">
@@ -488,7 +487,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>812153.6900000001</v>
+        <v>813787.01</v>
       </c>
     </row>
     <row r="5">
@@ -503,7 +502,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>1.7959239975</v>
+        <v>1.7960238975</v>
       </c>
     </row>
     <row r="6">
@@ -517,102 +516,7 @@
           <t>F0</t>
         </is>
       </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B8"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Row Name</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Measure Values</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>3rd_STG_Current</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>9.564949367500002e-07</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>2nd_STG_Current</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>1.428297495e-06</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>1st_STG_Current</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>7.80791412e-07</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Ground_AZCOMP</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>1.08070087e-05</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>OUTN_EXT_PRT</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>2.0037971025</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>OUTP_EXT_PRT</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>2.0067665425</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>VCM_AVDD</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>1.80382072</v>
-      </c>
+      <c r="C6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
added chip count for saving data, and modified .x;sx file
</commit_message>
<xml_diff>
--- a/DFT_6311_Result.xlsx
+++ b/DFT_6311_Result.xlsx
@@ -425,21 +425,26 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:D18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>Chip</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
           <t>Trimming</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Best Codes</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Closest Values</t>
         </is>
@@ -448,75 +453,308 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>chip1</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
           <t>VBGR_ADJ_TRIM</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>8E</t>
-        </is>
-      </c>
-      <c r="C2" t="n">
-        <v>1.80022254</v>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>AE</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>1.79742738</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>chip1</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
           <t>TSDN</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>9F</t>
-        </is>
-      </c>
-      <c r="C3" t="n">
-        <v>0.5422006655</v>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>0.5424838479999999</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
+          <t>chip1</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
           <t>FRO_CLOCK</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>E7</t>
-        </is>
-      </c>
-      <c r="C4" t="n">
-        <v>813787.01</v>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>F2</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>815174.2850000001</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
+          <t>chip1</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
           <t>BST_OCP_TRIM_reg1</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>70</t>
         </is>
       </c>
-      <c r="C5" t="n">
-        <v>1.7960238975</v>
+      <c r="D5" t="n">
+        <v>0.753176964</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
+          <t>chip1</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
           <t>BST_OCP_TRIM_reg2</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>D0</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr"/>
+      <c r="B7" t="inlineStr"/>
+      <c r="C7" t="inlineStr"/>
+      <c r="D7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>chip2</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>VBGR_ADJ_TRIM</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>AE</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>1.7974562525</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>chip2</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>TSDN</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>BF</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>0.54197220975</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>chip2</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>FRO_CLOCK</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>F2</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>815113.9899999998</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>chip2</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>BST_OCP_TRIM_reg1</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>0.7296092995</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>chip2</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>BST_OCP_TRIM_reg2</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>D0</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr"/>
+      <c r="B13" t="inlineStr"/>
+      <c r="C13" t="inlineStr"/>
+      <c r="D13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>chip3</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>VBGR_ADJ_TRIM</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>9E</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>1.7993927475</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>chip3</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>TSDN</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>0.542337132</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>chip3</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>FRO_CLOCK</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
         <is>
           <t>F0</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr"/>
+      <c r="D16" t="n">
+        <v>814786.0200000001</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>chip3</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>BST_OCP_TRIM_reg1</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>1.7937425275</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>chip3</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>BST_OCP_TRIM_reg2</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>F0</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>